<commit_message>
Rename the app to CoachAssist
README, package name and both Excel templates now use the CoachAssist name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GLR8JiJ3N4EjeuBHLa4v5D
</commit_message>
<xml_diff>
--- a/templates/BOMBA_Division_Sheet_Template.xlsx
+++ b/templates/BOMBA_Division_Sheet_Template.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
   <si>
-    <t xml:space="preserve">BOMBA Lineup Helper — Division Sheet</t>
+    <t xml:space="preserve">CoachAssist — Division Sheet</t>
   </si>
   <si>
     <t xml:space="preserve">Division</t>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">4. Yellow cells are for editing. Example rows show the format — replace them.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. In the app, an admin opens the division, taps Check, fixes anything listed, then taps Publish.</t>
+    <t xml:space="preserve">5. In CoachAssist, an admin opens the division, taps Check, fixes anything listed, then taps Publish.</t>
   </si>
   <si>
     <t xml:space="preserve">6. New coach emails must also be added to the Google Cloud test-user list (league admin).</t>
@@ -70,7 +70,7 @@
     <t xml:space="preserve">Coaches never see this Sheet. Each coach receives only their own team. Keep sharing on this file to admins and the division convenor.</t>
   </si>
   <si>
-    <t xml:space="preserve">Do not rename tabs or column headers — the app reads them.</t>
+    <t xml:space="preserve">Do not rename tabs or column headers — CoachAssist reads them.</t>
   </si>
   <si>
     <t xml:space="preserve">Teams</t>

</xml_diff>